<commit_message>
All except date and time
</commit_message>
<xml_diff>
--- a/test_data_generation.xlsx
+++ b/test_data_generation.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\TestDataGeneration\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E753FD1A-A020-4CF3-9D4A-862472D50327}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26791EA3-EA4C-42A0-BE1A-66A4CFFBFB01}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{1CEDB42C-FACB-4DBB-B373-A4400FAD661D}"/>
+    <workbookView xWindow="24" yWindow="24" windowWidth="23016" windowHeight="12336" xr2:uid="{1CEDB42C-FACB-4DBB-B373-A4400FAD661D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="55">
   <si>
     <t>Databasename</t>
   </si>
@@ -81,12 +82,12 @@
     <t>Country</t>
   </si>
   <si>
-    <t>PostCode</t>
-  </si>
-  <si>
     <t>Department_Id</t>
   </si>
   <si>
+    <t>number</t>
+  </si>
+  <si>
     <t>varchar</t>
   </si>
   <si>
@@ -102,9 +103,6 @@
     <t>postal code</t>
   </si>
   <si>
-    <t>PhoneNumber</t>
-  </si>
-  <si>
     <t>Primary Key</t>
   </si>
   <si>
@@ -117,9 +115,6 @@
     <t>Foreign Key</t>
   </si>
   <si>
-    <t>JoiningDate</t>
-  </si>
-  <si>
     <t>date</t>
   </si>
   <si>
@@ -150,9 +145,6 @@
     <t>Static_Value</t>
   </si>
   <si>
-    <t>US, NL,DE</t>
-  </si>
-  <si>
     <t>country</t>
   </si>
   <si>
@@ -193,6 +185,21 @@
   </si>
   <si>
     <t>ID</t>
+  </si>
+  <si>
+    <t>Joining_Date</t>
+  </si>
+  <si>
+    <t>Phone_Number</t>
+  </si>
+  <si>
+    <t>Post_Code</t>
+  </si>
+  <si>
+    <t>14,15,16,17</t>
+  </si>
+  <si>
+    <t>US, NL,DE,FR,IT</t>
   </si>
 </sst>
 </file>
@@ -549,7 +556,7 @@
   <cols>
     <col min="2" max="2" width="18.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19" customWidth="1"/>
+    <col min="4" max="4" width="10.77734375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="18.33203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13.5546875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="11.5546875" bestFit="1" customWidth="1"/>
@@ -566,7 +573,7 @@
         <v>7</v>
       </c>
       <c r="B1" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C1" t="s">
         <v>0</v>
@@ -587,22 +594,22 @@
         <v>9</v>
       </c>
       <c r="I1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="J1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="K1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="L1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="M1" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="N1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
@@ -610,42 +617,51 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="C2" t="s">
         <v>3</v>
       </c>
       <c r="D2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="E2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2" t="s">
         <v>16</v>
       </c>
-      <c r="F2" t="s">
-        <v>52</v>
-      </c>
       <c r="G2" t="s">
-        <v>23</v>
+        <v>22</v>
+      </c>
+      <c r="I2" t="s">
+        <v>53</v>
+      </c>
+      <c r="J2">
+        <v>1000</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
+      <c r="B3">
+        <v>4</v>
+      </c>
       <c r="C3" t="s">
         <v>3</v>
       </c>
       <c r="D3" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="E3" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F3" t="s">
         <v>17</v>
       </c>
       <c r="I3" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="L3">
         <v>50</v>
@@ -655,17 +671,20 @@
       <c r="A4">
         <v>3</v>
       </c>
+      <c r="B4">
+        <v>4</v>
+      </c>
       <c r="C4" t="s">
         <v>3</v>
       </c>
       <c r="D4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E4" t="s">
         <v>29</v>
       </c>
-      <c r="E4" t="s">
-        <v>31</v>
-      </c>
       <c r="F4" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.3">
@@ -673,7 +692,7 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>50</v>
+        <v>1000</v>
       </c>
       <c r="C5" t="s">
         <v>3</v>
@@ -685,13 +704,13 @@
         <v>5</v>
       </c>
       <c r="F5" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="G5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H5" t="s">
         <v>23</v>
-      </c>
-      <c r="H5" t="s">
-        <v>24</v>
       </c>
       <c r="J5">
         <v>100000</v>
@@ -704,6 +723,9 @@
       <c r="A6">
         <v>5</v>
       </c>
+      <c r="B6">
+        <v>1000</v>
+      </c>
       <c r="C6" t="s">
         <v>3</v>
       </c>
@@ -714,10 +736,10 @@
         <v>10</v>
       </c>
       <c r="F6" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="G6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="L6">
         <v>50</v>
@@ -727,6 +749,9 @@
       <c r="A7">
         <v>6</v>
       </c>
+      <c r="B7">
+        <v>1000</v>
+      </c>
       <c r="C7" t="s">
         <v>3</v>
       </c>
@@ -737,16 +762,10 @@
         <v>11</v>
       </c>
       <c r="F7" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="G7" t="s">
-        <v>51</v>
-      </c>
-      <c r="J7">
-        <v>3000</v>
-      </c>
-      <c r="K7">
-        <v>100000</v>
+        <v>48</v>
       </c>
       <c r="N7">
         <v>6</v>
@@ -756,6 +775,9 @@
       <c r="A8">
         <v>7</v>
       </c>
+      <c r="B8">
+        <v>1000</v>
+      </c>
       <c r="C8" t="s">
         <v>3</v>
       </c>
@@ -769,7 +791,7 @@
         <v>19</v>
       </c>
       <c r="H8" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="N8">
         <v>6</v>
@@ -779,6 +801,9 @@
       <c r="A9">
         <v>8</v>
       </c>
+      <c r="B9">
+        <v>1000</v>
+      </c>
       <c r="C9" t="s">
         <v>3</v>
       </c>
@@ -796,6 +821,9 @@
       <c r="A10">
         <v>9</v>
       </c>
+      <c r="B10">
+        <v>1000</v>
+      </c>
       <c r="C10" t="s">
         <v>3</v>
       </c>
@@ -806,22 +834,25 @@
         <v>14</v>
       </c>
       <c r="F10" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="G10" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I10" t="s">
-        <v>38</v>
+        <v>54</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
+      <c r="B11">
+        <v>1000</v>
+      </c>
       <c r="C11" t="s">
         <v>3</v>
       </c>
@@ -829,22 +860,25 @@
         <v>4</v>
       </c>
       <c r="E11" t="s">
+        <v>45</v>
+      </c>
+      <c r="F11" t="s">
+        <v>46</v>
+      </c>
+      <c r="G11" t="s">
         <v>48</v>
       </c>
-      <c r="F11" t="s">
-        <v>49</v>
-      </c>
       <c r="H11" t="s">
-        <v>24</v>
-      </c>
-      <c r="M11">
-        <v>6</v>
+        <v>23</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
+      <c r="B12">
+        <v>1000</v>
+      </c>
       <c r="C12" t="s">
         <v>3</v>
       </c>
@@ -852,7 +886,7 @@
         <v>4</v>
       </c>
       <c r="E12" t="s">
-        <v>15</v>
+        <v>52</v>
       </c>
       <c r="F12" t="s">
         <v>21</v>
@@ -866,7 +900,7 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>50</v>
+        <v>1000</v>
       </c>
       <c r="C13" t="s">
         <v>3</v>
@@ -875,13 +909,13 @@
         <v>4</v>
       </c>
       <c r="E13" t="s">
-        <v>22</v>
+        <v>51</v>
       </c>
       <c r="F13" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="G13" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.3">
@@ -889,7 +923,7 @@
         <v>13</v>
       </c>
       <c r="B14">
-        <v>50</v>
+        <v>1000</v>
       </c>
       <c r="C14" t="s">
         <v>3</v>
@@ -898,16 +932,16 @@
         <v>4</v>
       </c>
       <c r="E14" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F14" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="G14" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H14" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="N14">
         <v>1</v>
@@ -918,19 +952,19 @@
         <v>14</v>
       </c>
       <c r="B15">
+        <v>1000</v>
+      </c>
+      <c r="C15" t="s">
+        <v>3</v>
+      </c>
+      <c r="D15" t="s">
+        <v>4</v>
+      </c>
+      <c r="E15" t="s">
         <v>50</v>
       </c>
-      <c r="C15" t="s">
-        <v>3</v>
-      </c>
-      <c r="D15" t="s">
-        <v>4</v>
-      </c>
-      <c r="E15" t="s">
-        <v>27</v>
-      </c>
       <c r="F15" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.3">
@@ -938,22 +972,22 @@
         <v>15</v>
       </c>
       <c r="B16">
-        <v>12</v>
+        <v>150</v>
       </c>
       <c r="C16" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D16" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="E16" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="F16" t="s">
         <v>18</v>
       </c>
       <c r="G16" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="L16">
         <v>5</v>
@@ -963,20 +997,23 @@
       <c r="A17">
         <v>16</v>
       </c>
+      <c r="B17">
+        <v>150</v>
+      </c>
       <c r="C17" t="s">
+        <v>41</v>
+      </c>
+      <c r="D17" t="s">
+        <v>42</v>
+      </c>
+      <c r="E17" t="s">
         <v>44</v>
-      </c>
-      <c r="D17" t="s">
-        <v>45</v>
-      </c>
-      <c r="E17" t="s">
-        <v>47</v>
       </c>
       <c r="F17" t="s">
         <v>18</v>
       </c>
       <c r="G17" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="L17">
         <v>10</v>

</xml_diff>

<commit_message>
Committing date, time and datetime
Pending - Validations and locations
</commit_message>
<xml_diff>
--- a/test_data_generation.xlsx
+++ b/test_data_generation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\TestDataGeneration\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26791EA3-EA4C-42A0-BE1A-66A4CFFBFB01}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F57E426D-4282-4E3F-98CC-388F32ED25DB}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="24" yWindow="24" windowWidth="23016" windowHeight="12336" xr2:uid="{1CEDB42C-FACB-4DBB-B373-A4400FAD661D}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="57">
   <si>
     <t>Databasename</t>
   </si>
@@ -115,9 +115,6 @@
     <t>Foreign Key</t>
   </si>
   <si>
-    <t>date</t>
-  </si>
-  <si>
     <t>Department</t>
   </si>
   <si>
@@ -200,6 +197,15 @@
   </si>
   <si>
     <t>US, NL,DE,FR,IT</t>
+  </si>
+  <si>
+    <t>time</t>
+  </si>
+  <si>
+    <t>12:00:00</t>
+  </si>
+  <si>
+    <t>23:59:59</t>
   </si>
 </sst>
 </file>
@@ -235,8 +241,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -560,9 +567,8 @@
     <col min="5" max="5" width="18.33203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13.5546875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="11.5546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="23" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="30.88671875" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="18.109375" style="1" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="6.44140625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="8.33203125" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="16" bestFit="1" customWidth="1"/>
@@ -573,7 +579,7 @@
         <v>7</v>
       </c>
       <c r="B1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C1" t="s">
         <v>0</v>
@@ -594,22 +600,22 @@
         <v>9</v>
       </c>
       <c r="I1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="J1" t="s">
+        <v>32</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="K1" t="s">
-        <v>34</v>
-      </c>
       <c r="L1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="M1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="N1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
@@ -623,7 +629,7 @@
         <v>3</v>
       </c>
       <c r="D2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E2" t="s">
         <v>15</v>
@@ -635,9 +641,9 @@
         <v>22</v>
       </c>
       <c r="I2" t="s">
-        <v>53</v>
-      </c>
-      <c r="J2">
+        <v>52</v>
+      </c>
+      <c r="J2" s="1">
         <v>1000</v>
       </c>
     </row>
@@ -652,16 +658,16 @@
         <v>3</v>
       </c>
       <c r="D3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E3" t="s">
         <v>27</v>
-      </c>
-      <c r="E3" t="s">
-        <v>28</v>
       </c>
       <c r="F3" t="s">
         <v>17</v>
       </c>
       <c r="I3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L3">
         <v>50</v>
@@ -678,13 +684,13 @@
         <v>3</v>
       </c>
       <c r="D4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E4" t="s">
+        <v>28</v>
+      </c>
+      <c r="F4" t="s">
         <v>29</v>
-      </c>
-      <c r="F4" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.3">
@@ -704,7 +710,7 @@
         <v>5</v>
       </c>
       <c r="F5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G5" t="s">
         <v>22</v>
@@ -712,7 +718,7 @@
       <c r="H5" t="s">
         <v>23</v>
       </c>
-      <c r="J5">
+      <c r="J5" s="1">
         <v>100000</v>
       </c>
       <c r="L5">
@@ -736,7 +742,7 @@
         <v>10</v>
       </c>
       <c r="F6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G6" t="s">
         <v>24</v>
@@ -762,10 +768,10 @@
         <v>11</v>
       </c>
       <c r="F7" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G7" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N7">
         <v>6</v>
@@ -834,7 +840,7 @@
         <v>14</v>
       </c>
       <c r="F10" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G10" t="s">
         <v>24</v>
@@ -843,7 +849,7 @@
         <v>23</v>
       </c>
       <c r="I10" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
@@ -860,13 +866,13 @@
         <v>4</v>
       </c>
       <c r="E11" t="s">
+        <v>44</v>
+      </c>
+      <c r="F11" t="s">
         <v>45</v>
       </c>
-      <c r="F11" t="s">
-        <v>46</v>
-      </c>
       <c r="G11" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="H11" t="s">
         <v>23</v>
@@ -886,7 +892,7 @@
         <v>4</v>
       </c>
       <c r="E12" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F12" t="s">
         <v>21</v>
@@ -909,13 +915,13 @@
         <v>4</v>
       </c>
       <c r="E13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F13" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G13" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.3">
@@ -935,7 +941,7 @@
         <v>15</v>
       </c>
       <c r="F14" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G14" t="s">
         <v>25</v>
@@ -961,10 +967,19 @@
         <v>4</v>
       </c>
       <c r="E15" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F15" t="s">
-        <v>26</v>
+        <v>54</v>
+      </c>
+      <c r="G15" t="s">
+        <v>24</v>
+      </c>
+      <c r="J15" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="K15" s="1" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.3">
@@ -975,13 +990,13 @@
         <v>150</v>
       </c>
       <c r="C16" t="s">
+        <v>40</v>
+      </c>
+      <c r="D16" t="s">
         <v>41</v>
       </c>
-      <c r="D16" t="s">
+      <c r="E16" t="s">
         <v>42</v>
-      </c>
-      <c r="E16" t="s">
-        <v>43</v>
       </c>
       <c r="F16" t="s">
         <v>18</v>
@@ -1001,13 +1016,13 @@
         <v>150</v>
       </c>
       <c r="C17" t="s">
+        <v>40</v>
+      </c>
+      <c r="D17" t="s">
         <v>41</v>
       </c>
-      <c r="D17" t="s">
-        <v>42</v>
-      </c>
       <c r="E17" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F17" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
Nullable columns, lookups and unique lookups
</commit_message>
<xml_diff>
--- a/test_data_generation.xlsx
+++ b/test_data_generation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\TestDataGeneration\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70AB1758-BCF6-45D3-9E24-68E0ED16D8AB}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23F6C771-D201-4E99-996E-D56607EC1BF0}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="24" yWindow="24" windowWidth="23016" windowHeight="12336" xr2:uid="{1CEDB42C-FACB-4DBB-B373-A4400FAD661D}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="64">
   <si>
     <t>Databasename</t>
   </si>
@@ -214,6 +214,18 @@
   </si>
   <si>
     <t>Composite Key</t>
+  </si>
+  <si>
+    <t>Lookup</t>
+  </si>
+  <si>
+    <t>Manager</t>
+  </si>
+  <si>
+    <t>Unique Lookup</t>
+  </si>
+  <si>
+    <t>Manager_Country</t>
   </si>
 </sst>
 </file>
@@ -566,17 +578,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A143D004-ACBF-4C99-B125-08B251873804}">
-  <dimension ref="A1:N17"/>
+  <dimension ref="A1:N19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="1" max="1" width="5.44140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.33203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.77734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.6640625" customWidth="1"/>
-    <col min="9" max="9" width="30.88671875" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="18.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="23" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="10.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="6.44140625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="8.33203125" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="16" bestFit="1" customWidth="1"/>
@@ -659,9 +673,6 @@
       <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3">
-        <v>4</v>
-      </c>
       <c r="C3" t="s">
         <v>3</v>
       </c>
@@ -684,9 +695,6 @@
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
-      </c>
-      <c r="B4">
-        <v>4</v>
       </c>
       <c r="C4" t="s">
         <v>3</v>
@@ -740,9 +748,6 @@
       <c r="A6">
         <v>5</v>
       </c>
-      <c r="B6">
-        <v>100000</v>
-      </c>
       <c r="C6" t="s">
         <v>3</v>
       </c>
@@ -766,9 +771,6 @@
       <c r="A7">
         <v>6</v>
       </c>
-      <c r="B7">
-        <v>100000</v>
-      </c>
       <c r="C7" t="s">
         <v>3</v>
       </c>
@@ -782,7 +784,7 @@
         <v>16</v>
       </c>
       <c r="G7" t="s">
-        <v>24</v>
+        <v>60</v>
       </c>
       <c r="N7">
         <v>4</v>
@@ -792,9 +794,6 @@
       <c r="A8">
         <v>7</v>
       </c>
-      <c r="B8">
-        <v>100000</v>
-      </c>
       <c r="C8" t="s">
         <v>3</v>
       </c>
@@ -812,18 +811,12 @@
       </c>
       <c r="H8" t="s">
         <v>23</v>
-      </c>
-      <c r="N8">
-        <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
-      <c r="B9">
-        <v>100000</v>
-      </c>
       <c r="C9" t="s">
         <v>3</v>
       </c>
@@ -844,9 +837,6 @@
       <c r="A10">
         <v>9</v>
       </c>
-      <c r="B10">
-        <v>100000</v>
-      </c>
       <c r="C10" t="s">
         <v>3</v>
       </c>
@@ -870,9 +860,6 @@
       <c r="A11">
         <v>10</v>
       </c>
-      <c r="B11">
-        <v>100000</v>
-      </c>
       <c r="C11" t="s">
         <v>3</v>
       </c>
@@ -902,9 +889,6 @@
       <c r="A12">
         <v>11</v>
       </c>
-      <c r="B12">
-        <v>100000</v>
-      </c>
       <c r="C12" t="s">
         <v>3</v>
       </c>
@@ -919,18 +903,12 @@
       </c>
       <c r="G12" t="s">
         <v>24</v>
-      </c>
-      <c r="N12">
-        <v>6</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
-      <c r="B13">
-        <v>100000</v>
-      </c>
       <c r="C13" t="s">
         <v>3</v>
       </c>
@@ -951,9 +929,6 @@
       <c r="A14">
         <v>13</v>
       </c>
-      <c r="B14">
-        <v>100000</v>
-      </c>
       <c r="C14" t="s">
         <v>3</v>
       </c>
@@ -980,9 +955,6 @@
       <c r="A15">
         <v>14</v>
       </c>
-      <c r="B15">
-        <v>100000</v>
-      </c>
       <c r="C15" t="s">
         <v>3</v>
       </c>
@@ -1010,7 +982,7 @@
         <v>15</v>
       </c>
       <c r="B16">
-        <v>8</v>
+        <v>2500</v>
       </c>
       <c r="C16" t="s">
         <v>41</v>
@@ -1031,13 +1003,10 @@
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>16</v>
       </c>
-      <c r="B17">
-        <v>8</v>
-      </c>
       <c r="C17" t="s">
         <v>41</v>
       </c>
@@ -1055,6 +1024,58 @@
       </c>
       <c r="L17">
         <v>10</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18">
+        <v>15000</v>
+      </c>
+      <c r="C18" t="s">
+        <v>41</v>
+      </c>
+      <c r="D18" t="s">
+        <v>61</v>
+      </c>
+      <c r="E18" t="s">
+        <v>11</v>
+      </c>
+      <c r="F18" t="s">
+        <v>49</v>
+      </c>
+      <c r="G18" t="s">
+        <v>62</v>
+      </c>
+      <c r="N18">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="C19" t="s">
+        <v>41</v>
+      </c>
+      <c r="D19" t="s">
+        <v>61</v>
+      </c>
+      <c r="E19" t="s">
+        <v>63</v>
+      </c>
+      <c r="F19" t="s">
+        <v>18</v>
+      </c>
+      <c r="G19" t="s">
+        <v>60</v>
+      </c>
+      <c r="L19">
+        <v>10</v>
+      </c>
+      <c r="N19">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -1063,7 +1084,7 @@
       <formula1>"ID,char,varchar,number,decimal,postal code, phone number,state,state prefix,country,country prefix,date,datetime,time,city,city prefix,name,first name,last name"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G1048576" xr:uid="{E6A50AFB-0FA9-4A70-BCB0-10FF3B599256}">
-      <formula1>"Primary Key,Foreign Key,NA,Unique,Composite Key"</formula1>
+      <formula1>"Primary Key,Foreign Key,NA,Unique,Composite Key,Lookup,Unique Lookup"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2:H1048576" xr:uid="{5EDC5150-41FB-4B29-994C-2C6D52694202}">
       <formula1>"Y,N"</formula1>

</xml_diff>

<commit_message>
Implemented the function for DB connectionn
</commit_message>
<xml_diff>
--- a/test_data_generation.xlsx
+++ b/test_data_generation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\TestDataGeneration\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23F6C771-D201-4E99-996E-D56607EC1BF0}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{921FD9BC-9E79-4893-A940-5887A0E7CF00}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="24" yWindow="24" windowWidth="23016" windowHeight="12336" xr2:uid="{1CEDB42C-FACB-4DBB-B373-A4400FAD661D}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="62">
   <si>
     <t>Databasename</t>
   </si>
@@ -93,12 +93,6 @@
     <t>char</t>
   </si>
   <si>
-    <t>city prefix</t>
-  </si>
-  <si>
-    <t>state prefix</t>
-  </si>
-  <si>
     <t>postal code</t>
   </si>
   <si>
@@ -153,9 +147,6 @@
     <t>name</t>
   </si>
   <si>
-    <t>Marketing,IT,Sales,Security</t>
-  </si>
-  <si>
     <t>phone number</t>
   </si>
   <si>
@@ -195,24 +186,6 @@
     <t>Post_Code</t>
   </si>
   <si>
-    <t>14,15,16,17</t>
-  </si>
-  <si>
-    <t>2021-01-13</t>
-  </si>
-  <si>
-    <t>2005-01-01</t>
-  </si>
-  <si>
-    <t>1000</t>
-  </si>
-  <si>
-    <t>12000</t>
-  </si>
-  <si>
-    <t>9999999</t>
-  </si>
-  <si>
     <t>Composite Key</t>
   </si>
   <si>
@@ -226,6 +199,27 @@
   </si>
   <si>
     <t>Manager_Country</t>
+  </si>
+  <si>
+    <t>state</t>
+  </si>
+  <si>
+    <t>address</t>
+  </si>
+  <si>
+    <t>Joining_time</t>
+  </si>
+  <si>
+    <t>time</t>
+  </si>
+  <si>
+    <t>Gender</t>
+  </si>
+  <si>
+    <t>M,F,NB</t>
+  </si>
+  <si>
+    <t>country prefix</t>
   </si>
 </sst>
 </file>
@@ -578,7 +572,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A143D004-ACBF-4C99-B125-08B251873804}">
-  <dimension ref="A1:N19"/>
+  <dimension ref="A1:N21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.44140625" bestFit="1" customWidth="1"/>
@@ -601,7 +595,7 @@
         <v>7</v>
       </c>
       <c r="B1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C1" t="s">
         <v>0</v>
@@ -622,22 +616,22 @@
         <v>9</v>
       </c>
       <c r="I1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="J1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="L1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="M1" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="N1" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
@@ -645,13 +639,13 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>4</v>
+        <v>100000</v>
       </c>
       <c r="C2" t="s">
         <v>3</v>
       </c>
       <c r="D2" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E2" t="s">
         <v>15</v>
@@ -660,13 +654,7 @@
         <v>16</v>
       </c>
       <c r="G2" t="s">
-        <v>22</v>
-      </c>
-      <c r="I2" t="s">
-        <v>53</v>
-      </c>
-      <c r="J2" s="1">
-        <v>1000</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.3">
@@ -677,19 +665,19 @@
         <v>3</v>
       </c>
       <c r="D3" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E3" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="F3" t="s">
         <v>17</v>
       </c>
-      <c r="I3" t="s">
-        <v>39</v>
+      <c r="G3" t="s">
+        <v>45</v>
       </c>
       <c r="L3">
-        <v>50</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
@@ -700,13 +688,19 @@
         <v>3</v>
       </c>
       <c r="D4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E4" t="s">
         <v>27</v>
       </c>
-      <c r="E4" t="s">
-        <v>29</v>
-      </c>
       <c r="F4" t="s">
-        <v>30</v>
+        <v>28</v>
+      </c>
+      <c r="G4" t="s">
+        <v>22</v>
+      </c>
+      <c r="H4" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.3">
@@ -714,7 +708,7 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>100000</v>
+        <v>10000</v>
       </c>
       <c r="C5" t="s">
         <v>3</v>
@@ -726,19 +720,10 @@
         <v>5</v>
       </c>
       <c r="F5" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="G5" t="s">
-        <v>22</v>
-      </c>
-      <c r="H5" t="s">
-        <v>23</v>
-      </c>
-      <c r="J5" s="1">
-        <v>100000</v>
-      </c>
-      <c r="K5" s="1" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="L5">
         <v>6</v>
@@ -758,10 +743,10 @@
         <v>10</v>
       </c>
       <c r="F6" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="G6" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="L6">
         <v>50</v>
@@ -784,7 +769,7 @@
         <v>16</v>
       </c>
       <c r="G7" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="N7">
         <v>4</v>
@@ -804,13 +789,13 @@
         <v>12</v>
       </c>
       <c r="F8" t="s">
-        <v>19</v>
+        <v>56</v>
       </c>
       <c r="G8" t="s">
-        <v>59</v>
+        <v>22</v>
       </c>
       <c r="H8" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
@@ -827,10 +812,10 @@
         <v>13</v>
       </c>
       <c r="F9" t="s">
-        <v>20</v>
+        <v>55</v>
       </c>
       <c r="G9" t="s">
-        <v>59</v>
+        <v>22</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
@@ -847,13 +832,10 @@
         <v>14</v>
       </c>
       <c r="F10" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="G10" t="s">
-        <v>59</v>
-      </c>
-      <c r="H10" t="s">
-        <v>23</v>
+        <v>50</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
@@ -867,22 +849,16 @@
         <v>4</v>
       </c>
       <c r="E11" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="F11" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="G11" t="s">
-        <v>24</v>
-      </c>
-      <c r="H11" t="s">
-        <v>23</v>
-      </c>
-      <c r="J11" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="K11" s="1" t="s">
-        <v>57</v>
+        <v>22</v>
+      </c>
+      <c r="M11">
+        <v>4</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
@@ -896,13 +872,13 @@
         <v>4</v>
       </c>
       <c r="E12" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="F12" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="G12" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.3">
@@ -916,13 +892,13 @@
         <v>4</v>
       </c>
       <c r="E13" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="F13" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="G13" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.3">
@@ -939,12 +915,9 @@
         <v>15</v>
       </c>
       <c r="F14" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="G14" t="s">
-        <v>25</v>
-      </c>
-      <c r="H14" t="s">
         <v>23</v>
       </c>
       <c r="N14">
@@ -962,68 +935,56 @@
         <v>4</v>
       </c>
       <c r="E15" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="F15" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="G15" t="s">
-        <v>24</v>
-      </c>
-      <c r="J15" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="K15" s="1" t="s">
-        <v>54</v>
+        <v>22</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>15</v>
       </c>
-      <c r="B16">
-        <v>2500</v>
-      </c>
       <c r="C16" t="s">
-        <v>41</v>
+        <v>3</v>
       </c>
       <c r="D16" t="s">
-        <v>42</v>
+        <v>4</v>
       </c>
       <c r="E16" t="s">
-        <v>43</v>
+        <v>57</v>
       </c>
       <c r="F16" t="s">
-        <v>49</v>
-      </c>
-      <c r="G16" t="s">
-        <v>22</v>
-      </c>
-      <c r="L16">
-        <v>5</v>
+        <v>58</v>
       </c>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>16</v>
       </c>
+      <c r="B17">
+        <v>800</v>
+      </c>
       <c r="C17" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="D17" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="E17" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="F17" t="s">
-        <v>18</v>
+        <v>46</v>
       </c>
       <c r="G17" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="L17">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.3">
@@ -1031,57 +992,106 @@
         <v>17</v>
       </c>
       <c r="B18">
-        <v>15000</v>
+        <v>800</v>
       </c>
       <c r="C18" t="s">
+        <v>38</v>
+      </c>
+      <c r="D18" t="s">
+        <v>39</v>
+      </c>
+      <c r="E18" t="s">
         <v>41</v>
       </c>
-      <c r="D18" t="s">
-        <v>61</v>
-      </c>
-      <c r="E18" t="s">
-        <v>11</v>
-      </c>
       <c r="F18" t="s">
-        <v>49</v>
+        <v>18</v>
       </c>
       <c r="G18" t="s">
-        <v>62</v>
-      </c>
-      <c r="N18">
-        <v>6</v>
+        <v>22</v>
+      </c>
+      <c r="L18">
+        <v>10</v>
       </c>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>18</v>
       </c>
+      <c r="B19">
+        <v>100</v>
+      </c>
       <c r="C19" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="D19" t="s">
+        <v>52</v>
+      </c>
+      <c r="E19" t="s">
+        <v>11</v>
+      </c>
+      <c r="F19" t="s">
+        <v>46</v>
+      </c>
+      <c r="G19" t="s">
+        <v>53</v>
+      </c>
+      <c r="N19">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20">
+        <v>100</v>
+      </c>
+      <c r="C20" t="s">
+        <v>38</v>
+      </c>
+      <c r="D20" t="s">
+        <v>52</v>
+      </c>
+      <c r="E20" t="s">
+        <v>54</v>
+      </c>
+      <c r="F20" t="s">
         <v>61</v>
       </c>
-      <c r="E19" t="s">
-        <v>63</v>
-      </c>
-      <c r="F19" t="s">
+      <c r="G20" t="s">
+        <v>22</v>
+      </c>
+      <c r="L20">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="C21" t="s">
+        <v>38</v>
+      </c>
+      <c r="D21" t="s">
+        <v>52</v>
+      </c>
+      <c r="E21" t="s">
+        <v>59</v>
+      </c>
+      <c r="F21" t="s">
         <v>18</v>
       </c>
-      <c r="G19" t="s">
+      <c r="H21" t="s">
+        <v>21</v>
+      </c>
+      <c r="I21" t="s">
         <v>60</v>
-      </c>
-      <c r="L19">
-        <v>10</v>
-      </c>
-      <c r="N19">
-        <v>9</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F1048576" xr:uid="{F90728EC-FB1F-4606-ADDB-38D448E29600}">
-      <formula1>"ID,char,varchar,number,decimal,postal code, phone number,state,state prefix,country,country prefix,date,datetime,time,city,city prefix,name,first name,last name"</formula1>
+      <formula1>"ID,address,char,varchar,number,decimal,postal code, phone number,state,country,country prefix,date,datetime,time,city,city prefix,name,first name,last name"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G1048576" xr:uid="{E6A50AFB-0FA9-4A70-BCB0-10FF3B599256}">
       <formula1>"Primary Key,Foreign Key,NA,Unique,Composite Key,Lookup,Unique Lookup"</formula1>

</xml_diff>